<commit_message>
Modificato Lista parti: mancava L1
</commit_message>
<xml_diff>
--- a/ESECUTIVI/LP25-336-0_ASSY00_Rev00.xlsx
+++ b/ESECUTIVI/LP25-336-0_ASSY00_Rev00.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documents\Data\Progetti-GIT\HW\pcb-25-336\ESECUTIVI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A90AFC7-8362-4B47-AA43-20D207CC59AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB2CA06D-922F-4D6A-9DB0-9AFADC0AE98F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{6B4F9678-F329-48FB-B22C-A9FC5D2A2934}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6B4F9678-F329-48FB-B22C-A9FC5D2A2934}"/>
   </bookViews>
   <sheets>
     <sheet name="25-336-0" sheetId="1" r:id="rId1"/>
     <sheet name="Revision" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'25-336-0'!$A$1:$J$78</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'25-336-0'!$A$1:$J$79</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="422">
   <si>
     <t>Pos.</t>
   </si>
@@ -1269,6 +1269,34 @@
 - R35:  (can bus) non montare.
 - Test points: non montare, si usano solo le piazzole
 - J6: non momtare. E' una predisposizione per una scheda aggiuntiva per la tensione di griglia</t>
+  </si>
+  <si>
+    <t>CC1206JRX7R9BB104</t>
+  </si>
+  <si>
+    <t>603-C1206JRX7R9BB104</t>
+  </si>
+  <si>
+    <t>37a</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>37b</t>
+  </si>
+  <si>
+    <t>Induttori accoppiati WE-CFWI Cpld Flatwr 
+10uH 13A 13.9mOhms</t>
+  </si>
+  <si>
+    <t>10uH</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 710-74485540101</t>
+  </si>
+  <si>
+    <t>WE-74485540101</t>
   </si>
 </sst>
 </file>
@@ -2302,12 +2330,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{262EEB21-1FA5-479A-A8B0-1CAA3EE72DB4}">
-  <dimension ref="A1:K79"/>
+  <dimension ref="A1:K80"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.42578125" style="2" customWidth="1"/>
     <col min="2" max="2" width="5.5703125" style="14" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="1"/>
+    <col min="3" max="3" width="51" style="1" customWidth="1"/>
     <col min="4" max="4" width="49" style="1" customWidth="1"/>
     <col min="5" max="5" width="25.140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="24.42578125" style="1" customWidth="1"/>
@@ -2473,14 +2501,14 @@
       <c r="E6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="11">
-        <v>885012214005</v>
+      <c r="F6" s="11" t="s">
+        <v>413</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>315</v>
+        <v>414</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>289</v>
+        <v>211</v>
       </c>
       <c r="I6" s="9"/>
       <c r="J6" s="9" t="s">
@@ -3412,7 +3440,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="8">
         <v>35</v>
       </c>
@@ -3473,221 +3501,221 @@
       </c>
     </row>
     <row r="39" spans="1:11" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A39" s="8">
-        <v>37</v>
+      <c r="A39" s="8" t="s">
+        <v>415</v>
       </c>
       <c r="B39" s="13">
         <v>1</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>157</v>
+        <v>416</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>158</v>
+        <v>418</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="F39" s="9" t="s">
-        <v>159</v>
+        <v>419</v>
+      </c>
+      <c r="F39" s="9">
+        <v>74485540101</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>327</v>
+        <v>420</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="I39" s="9" t="s">
-        <v>159</v>
+        <v>289</v>
+      </c>
+      <c r="I39" s="9">
+        <v>74485540101</v>
       </c>
       <c r="J39" s="9" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" ht="57" x14ac:dyDescent="0.25">
-      <c r="A40" s="8">
-        <v>38</v>
+        <v>421</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A40" s="8" t="s">
+        <v>417</v>
       </c>
       <c r="B40" s="13">
         <v>1</v>
       </c>
       <c r="C40" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F40" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="G40" s="15" t="s">
+        <v>327</v>
+      </c>
+      <c r="H40" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="I40" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="J40" s="9" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="57" x14ac:dyDescent="0.25">
+      <c r="A41" s="8">
+        <v>38</v>
+      </c>
+      <c r="B41" s="13">
+        <v>1</v>
+      </c>
+      <c r="C41" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="D40" s="9" t="s">
+      <c r="D41" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="E40" s="9" t="s">
+      <c r="E41" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="F40" s="9" t="s">
+      <c r="F41" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="G40" s="25" t="s">
+      <c r="G41" s="25" t="s">
         <v>328</v>
       </c>
-      <c r="H40" s="9" t="s">
+      <c r="H41" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="I40" s="9" t="s">
+      <c r="I41" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="J40" s="9" t="s">
+      <c r="J41" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="K40" s="1" t="s">
+      <c r="K41" s="1" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A41" s="8">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" s="8">
         <v>39</v>
       </c>
-      <c r="B41" s="13">
+      <c r="B42" s="13">
         <v>2</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C42" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="D41" s="9" t="s">
+      <c r="D42" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="E41" s="9" t="s">
+      <c r="E42" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="F41" s="9" t="s">
+      <c r="F42" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="G41" s="9" t="s">
+      <c r="G42" s="9" t="s">
         <v>329</v>
       </c>
-      <c r="H41" s="9" t="s">
+      <c r="H42" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="I41" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="J41" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" ht="85.5" x14ac:dyDescent="0.25">
-      <c r="A42" s="8">
+      <c r="I42" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J42" s="9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="85.5" x14ac:dyDescent="0.25">
+      <c r="A43" s="8">
         <v>40</v>
       </c>
-      <c r="B42" s="13">
+      <c r="B43" s="13">
         <v>11</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C43" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="D42" s="9" t="s">
+      <c r="D43" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="E42" s="9" t="s">
+      <c r="E43" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="F42" s="9" t="s">
+      <c r="F43" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="G42" s="9" t="s">
+      <c r="G43" s="9" t="s">
         <v>380</v>
       </c>
-      <c r="H42" s="9" t="s">
+      <c r="H43" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="I42" s="9" t="s">
+      <c r="I43" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="J42" s="9" t="s">
+      <c r="J43" s="9" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="8">
+    <row r="44" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A44" s="8">
         <v>41</v>
       </c>
-      <c r="B43" s="13">
+      <c r="B44" s="13">
         <v>1</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C44" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="D43" s="9" t="s">
+      <c r="D44" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="E43" s="9" t="s">
+      <c r="E44" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="F43" s="9" t="s">
+      <c r="F44" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="G43" s="9" t="s">
+      <c r="G44" s="9" t="s">
         <v>379</v>
       </c>
-      <c r="H43" s="9" t="s">
+      <c r="H44" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="I43" s="9" t="s">
+      <c r="I44" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="J43" s="9" t="s">
+      <c r="J44" s="9" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="8">
+    <row r="45" spans="1:11" ht="42.75" x14ac:dyDescent="0.25">
+      <c r="A45" s="8">
         <v>42</v>
       </c>
-      <c r="B44" s="13">
+      <c r="B45" s="13">
         <v>5</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="C45" s="9" t="s">
         <v>183</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="E44" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>373</v>
-      </c>
-      <c r="G44" s="9" t="s">
-        <v>374</v>
-      </c>
-      <c r="H44" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="I44" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="J44" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A45" s="8">
-        <v>43</v>
-      </c>
-      <c r="B45" s="13">
-        <v>1</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>187</v>
       </c>
       <c r="D45" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="G45" s="9" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="H45" s="9" t="s">
         <v>186</v>
@@ -3699,27 +3727,27 @@
         <v>14</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="8">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B46" s="13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D46" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>343</v>
+        <v>371</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>344</v>
+        <v>372</v>
       </c>
       <c r="H46" s="9" t="s">
         <v>186</v>
@@ -3731,27 +3759,27 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A47" s="8">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B47" s="13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D47" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>369</v>
+        <v>343</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>370</v>
+        <v>344</v>
       </c>
       <c r="H47" s="9" t="s">
         <v>186</v>
@@ -3763,27 +3791,27 @@
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="57" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="8">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B48" s="13">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D48" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>330</v>
+        <v>369</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>331</v>
+        <v>370</v>
       </c>
       <c r="H48" s="9" t="s">
         <v>186</v>
@@ -3795,91 +3823,91 @@
         <v>14</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" ht="57" x14ac:dyDescent="0.25">
       <c r="A49" s="8">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B49" s="13">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>350</v>
+        <v>330</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>378</v>
+        <v>331</v>
       </c>
       <c r="H49" s="9" t="s">
-        <v>96</v>
+        <v>186</v>
       </c>
       <c r="I49" s="9" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="J49" s="9" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="8">
+        <v>47</v>
+      </c>
+      <c r="B50" s="13">
+        <v>2</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="F50" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="G50" s="9" t="s">
+        <v>378</v>
+      </c>
+      <c r="H50" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="I50" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J50" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" s="8">
         <v>48</v>
       </c>
-      <c r="B50" s="13">
+      <c r="B51" s="13">
         <v>1</v>
       </c>
-      <c r="C50" s="9" t="s">
+      <c r="C51" s="9" t="s">
         <v>198</v>
-      </c>
-      <c r="D50" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="E50" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="F50" s="9" t="s">
-        <v>349</v>
-      </c>
-      <c r="G50" s="9" t="s">
-        <v>377</v>
-      </c>
-      <c r="H50" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="I50" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="J50" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A51" s="8">
-        <v>49</v>
-      </c>
-      <c r="B51" s="13">
-        <v>4</v>
-      </c>
-      <c r="C51" s="9" t="s">
-        <v>200</v>
       </c>
       <c r="D51" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>342</v>
+        <v>377</v>
       </c>
       <c r="H51" s="9" t="s">
         <v>186</v>
@@ -3891,27 +3919,27 @@
         <v>14</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A52" s="8">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B52" s="13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D52" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>368</v>
+        <v>341</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>367</v>
+        <v>342</v>
       </c>
       <c r="H52" s="9" t="s">
         <v>186</v>
@@ -3925,25 +3953,25 @@
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="8">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B53" s="13">
         <v>1</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D53" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="H53" s="9" t="s">
         <v>186</v>
@@ -3955,91 +3983,91 @@
         <v>14</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="8">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B54" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>207</v>
+        <v>184</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>209</v>
+        <v>365</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>210</v>
+        <v>366</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>211</v>
+        <v>186</v>
       </c>
       <c r="I54" s="9" t="s">
-        <v>212</v>
+        <v>14</v>
       </c>
       <c r="J54" s="9" t="s">
-        <v>212</v>
+        <v>14</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A55" s="8">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B55" s="13">
         <v>2</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>184</v>
+        <v>207</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>363</v>
+        <v>209</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>364</v>
+        <v>210</v>
       </c>
       <c r="H55" s="9" t="s">
-        <v>186</v>
+        <v>211</v>
       </c>
       <c r="I55" s="9" t="s">
-        <v>14</v>
+        <v>212</v>
       </c>
       <c r="J55" s="9" t="s">
-        <v>14</v>
+        <v>212</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A56" s="8">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B56" s="13">
         <v>2</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D56" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="H56" s="9" t="s">
         <v>186</v>
@@ -4053,25 +4081,25 @@
     </row>
     <row r="57" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A57" s="8">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B57" s="13">
         <v>2</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D57" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>339</v>
+        <v>361</v>
       </c>
       <c r="G57" s="9" t="s">
-        <v>340</v>
+        <v>362</v>
       </c>
       <c r="H57" s="9" t="s">
         <v>186</v>
@@ -4085,25 +4113,25 @@
     </row>
     <row r="58" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A58" s="8">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B58" s="13">
         <v>2</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D58" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>359</v>
+        <v>339</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>360</v>
+        <v>340</v>
       </c>
       <c r="H58" s="9" t="s">
         <v>186</v>
@@ -4115,27 +4143,27 @@
         <v>14</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A59" s="8">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B59" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D59" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F59" s="9" t="s">
-        <v>332</v>
+        <v>359</v>
       </c>
       <c r="G59" s="9" t="s">
-        <v>376</v>
+        <v>360</v>
       </c>
       <c r="H59" s="9" t="s">
         <v>186</v>
@@ -4147,27 +4175,27 @@
         <v>14</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="8">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B60" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>402</v>
+        <v>221</v>
       </c>
       <c r="D60" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>334</v>
+        <v>376</v>
       </c>
       <c r="H60" s="9" t="s">
         <v>186</v>
@@ -4179,94 +4207,94 @@
         <v>14</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A61" s="20" t="s">
+    <row r="61" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A61" s="8">
+        <v>58</v>
+      </c>
+      <c r="B61" s="13">
+        <v>2</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>402</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="E61" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="F61" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="G61" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="H61" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="I61" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J61" s="9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A62" s="20" t="s">
         <v>403</v>
       </c>
-      <c r="B61" s="21">
+      <c r="B62" s="21">
         <v>1</v>
       </c>
-      <c r="C61" s="22" t="s">
+      <c r="C62" s="22" t="s">
         <v>404</v>
       </c>
-      <c r="D61" s="22" t="s">
+      <c r="D62" s="22" t="s">
         <v>184</v>
       </c>
-      <c r="E61" s="22" t="s">
+      <c r="E62" s="22" t="s">
         <v>223</v>
       </c>
-      <c r="F61" s="22" t="s">
+      <c r="F62" s="22" t="s">
         <v>333</v>
       </c>
-      <c r="G61" s="22" t="s">
+      <c r="G62" s="22" t="s">
         <v>334</v>
       </c>
-      <c r="H61" s="22" t="s">
+      <c r="H62" s="22" t="s">
         <v>186</v>
       </c>
-      <c r="I61" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="J61" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="K61" s="23" t="s">
+      <c r="I62" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="J62" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="K62" s="23" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A62" s="8">
+    <row r="63" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A63" s="8">
         <v>59</v>
       </c>
-      <c r="B62" s="13">
+      <c r="B63" s="13">
         <v>3</v>
       </c>
-      <c r="C62" s="9" t="s">
+      <c r="C63" s="9" t="s">
         <v>224</v>
-      </c>
-      <c r="D62" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="E62" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="F62" s="9" t="s">
-        <v>335</v>
-      </c>
-      <c r="G62" s="9" t="s">
-        <v>336</v>
-      </c>
-      <c r="H62" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="I62" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="J62" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A63" s="8">
-        <v>60</v>
-      </c>
-      <c r="B63" s="13">
-        <v>1</v>
-      </c>
-      <c r="C63" s="9" t="s">
-        <v>226</v>
       </c>
       <c r="D63" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F63" s="9" t="s">
-        <v>345</v>
+        <v>335</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>346</v>
+        <v>336</v>
       </c>
       <c r="H63" s="9" t="s">
         <v>186</v>
@@ -4280,121 +4308,121 @@
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="8">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B64" s="13">
         <v>1</v>
       </c>
       <c r="C64" s="9" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>229</v>
+        <v>184</v>
       </c>
       <c r="E64" s="9" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
       <c r="G64" s="9" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="H64" s="9" t="s">
         <v>186</v>
       </c>
       <c r="I64" s="9" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="J64" s="9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="8">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B65" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C65" s="9" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>232</v>
+        <v>214</v>
       </c>
       <c r="F65" s="9" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="H65" s="9" t="s">
         <v>186</v>
       </c>
       <c r="I65" s="9" t="s">
-        <v>233</v>
+        <v>23</v>
       </c>
       <c r="J65" s="9" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A66" s="8">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B66" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C66" s="9" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>184</v>
+        <v>231</v>
       </c>
       <c r="E66" s="9" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="G66" s="9" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="H66" s="9" t="s">
         <v>186</v>
       </c>
       <c r="I66" s="9" t="s">
-        <v>14</v>
+        <v>233</v>
       </c>
       <c r="J66" s="9" t="s">
-        <v>14</v>
+        <v>233</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="8">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B67" s="13">
         <v>1</v>
       </c>
       <c r="C67" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D67" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="F67" s="9" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="H67" s="9" t="s">
         <v>186</v>
@@ -4406,27 +4434,27 @@
         <v>14</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="71.25" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="8">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B68" s="13">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C68" s="9" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D68" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="H68" s="9" t="s">
         <v>186</v>
@@ -4440,25 +4468,25 @@
     </row>
     <row r="69" spans="1:11" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A69" s="8">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B69" s="13">
         <v>7</v>
       </c>
       <c r="C69" s="9" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D69" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="F69" s="9" t="s">
-        <v>337</v>
+        <v>351</v>
       </c>
       <c r="G69" s="9" t="s">
-        <v>338</v>
+        <v>352</v>
       </c>
       <c r="H69" s="9" t="s">
         <v>186</v>
@@ -4471,319 +4499,351 @@
       </c>
     </row>
     <row r="70" spans="1:11" ht="71.25" x14ac:dyDescent="0.25">
-      <c r="A70" s="20">
+      <c r="A70" s="8">
+        <v>66</v>
+      </c>
+      <c r="B70" s="13">
+        <v>7</v>
+      </c>
+      <c r="C70" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="E70" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="F70" s="9" t="s">
+        <v>337</v>
+      </c>
+      <c r="G70" s="9" t="s">
+        <v>338</v>
+      </c>
+      <c r="H70" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="I70" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J70" s="9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" ht="71.25" x14ac:dyDescent="0.25">
+      <c r="A71" s="20">
         <v>67</v>
       </c>
-      <c r="B70" s="21">
+      <c r="B71" s="21">
         <v>7</v>
       </c>
-      <c r="C70" s="22" t="s">
+      <c r="C71" s="22" t="s">
         <v>242</v>
       </c>
-      <c r="D70" s="22" t="s">
+      <c r="D71" s="22" t="s">
         <v>243</v>
       </c>
-      <c r="E70" s="22" t="s">
+      <c r="E71" s="22" t="s">
         <v>244</v>
       </c>
-      <c r="F70" s="22" t="s">
+      <c r="F71" s="22" t="s">
         <v>244</v>
       </c>
-      <c r="G70" s="22" t="s">
+      <c r="G71" s="22" t="s">
         <v>375</v>
       </c>
-      <c r="H70" s="26" t="b">
+      <c r="H71" s="26" t="b">
         <v>1</v>
       </c>
-      <c r="I70" s="22" t="s">
+      <c r="I71" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="J70" s="22" t="s">
+      <c r="J71" s="22" t="s">
         <v>245</v>
       </c>
-      <c r="K70" s="23" t="s">
+      <c r="K71" s="23" t="s">
         <v>308</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A71" s="8">
-        <v>68</v>
-      </c>
-      <c r="B71" s="13">
-        <v>1</v>
-      </c>
-      <c r="C71" s="9" t="s">
-        <v>246</v>
-      </c>
-      <c r="D71" s="9" t="s">
-        <v>247</v>
-      </c>
-      <c r="E71" s="9" t="s">
-        <v>248</v>
-      </c>
-      <c r="F71" s="9" t="s">
-        <v>248</v>
-      </c>
-      <c r="G71" s="9" t="s">
-        <v>393</v>
-      </c>
-      <c r="H71" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="I71" s="9"/>
-      <c r="J71" s="9" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="72" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A72" s="8">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B72" s="13">
         <v>1</v>
       </c>
       <c r="C72" s="9" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="E72" s="9" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="F72" s="9" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="H72" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="I72" s="9" t="s">
-        <v>254</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="I72" s="9"/>
       <c r="J72" s="9" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="73" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A73" s="8">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B73" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C73" s="9" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="F73" s="9" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>96</v>
+        <v>253</v>
       </c>
       <c r="I73" s="9" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J73" s="9" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
     </row>
     <row r="74" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A74" s="8">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B74" s="13">
         <v>2</v>
       </c>
       <c r="C74" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="D74" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="E74" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="F74" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="G74" s="9" t="s">
+        <v>395</v>
+      </c>
+      <c r="H74" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="I74" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="J74" s="9" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A75" s="8">
+        <v>71</v>
+      </c>
+      <c r="B75" s="13">
+        <v>2</v>
+      </c>
+      <c r="C75" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="D74" s="9" t="s">
+      <c r="D75" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="E74" s="9" t="s">
+      <c r="E75" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="F74" s="9" t="s">
+      <c r="F75" s="9" t="s">
         <v>396</v>
       </c>
-      <c r="G74" s="9" t="s">
+      <c r="G75" s="9" t="s">
         <v>406</v>
       </c>
-      <c r="H74" s="9" t="s">
+      <c r="H75" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="I74" s="9"/>
-      <c r="J74" s="9" t="s">
+      <c r="I75" s="9"/>
+      <c r="J75" s="9" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A75" s="8">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A76" s="8">
         <v>72</v>
-      </c>
-      <c r="B75" s="13">
-        <v>1</v>
-      </c>
-      <c r="C75" s="9" t="s">
-        <v>266</v>
-      </c>
-      <c r="D75" s="9" t="s">
-        <v>267</v>
-      </c>
-      <c r="E75" s="9" t="s">
-        <v>268</v>
-      </c>
-      <c r="F75" s="9" t="s">
-        <v>268</v>
-      </c>
-      <c r="G75" s="9" t="s">
-        <v>397</v>
-      </c>
-      <c r="H75" s="9" t="s">
-        <v>269</v>
-      </c>
-      <c r="I75" s="9" t="s">
-        <v>270</v>
-      </c>
-      <c r="J75" s="9" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A76" s="8">
-        <v>73</v>
       </c>
       <c r="B76" s="13">
         <v>1</v>
       </c>
       <c r="C76" s="9" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="E76" s="9" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="F76" s="9" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="G76" s="9" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="H76" s="9" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="I76" s="9" t="s">
-        <v>139</v>
+        <v>270</v>
       </c>
       <c r="J76" s="9" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A77" s="8">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B77" s="13">
         <v>1</v>
       </c>
       <c r="C77" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="D77" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="E77" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="F77" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="G77" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="H77" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="I77" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="J77" s="9" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A78" s="8">
+        <v>74</v>
+      </c>
+      <c r="B78" s="13">
+        <v>1</v>
+      </c>
+      <c r="C78" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="D77" s="9" t="s">
+      <c r="D78" s="9" t="s">
         <v>278</v>
       </c>
-      <c r="E77" s="9" t="s">
+      <c r="E78" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="F77" s="9" t="s">
+      <c r="F78" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="G77" s="9" t="s">
+      <c r="G78" s="9" t="s">
         <v>399</v>
       </c>
-      <c r="H77" s="9" t="s">
+      <c r="H78" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="I77" s="9" t="s">
+      <c r="I78" s="9" t="s">
         <v>280</v>
       </c>
-      <c r="J77" s="9" t="s">
+      <c r="J78" s="9" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A78" s="16">
+    <row r="79" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A79" s="16">
         <v>75</v>
       </c>
-      <c r="B78" s="17">
+      <c r="B79" s="17">
         <v>1</v>
       </c>
-      <c r="C78" s="18" t="s">
+      <c r="C79" s="18" t="s">
         <v>282</v>
       </c>
-      <c r="D78" s="18" t="s">
+      <c r="D79" s="18" t="s">
         <v>283</v>
       </c>
-      <c r="E78" s="18" t="s">
+      <c r="E79" s="18" t="s">
         <v>284</v>
       </c>
-      <c r="F78" s="18" t="s">
+      <c r="F79" s="18" t="s">
         <v>284</v>
       </c>
-      <c r="G78" s="18" t="s">
+      <c r="G79" s="18" t="s">
         <v>400</v>
       </c>
-      <c r="H78" s="18" t="s">
+      <c r="H79" s="18" t="s">
         <v>285</v>
       </c>
-      <c r="I78" s="18" t="s">
+      <c r="I79" s="18" t="s">
         <v>286</v>
       </c>
-      <c r="J78" s="18" t="s">
+      <c r="J79" s="18" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A79" s="8">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A80" s="8">
         <v>76</v>
       </c>
-      <c r="B79" s="13">
+      <c r="B80" s="13">
         <v>1</v>
       </c>
-      <c r="C79" s="9" t="s">
+      <c r="C80" s="9" t="s">
         <v>294</v>
       </c>
-      <c r="D79" s="9" t="s">
+      <c r="D80" s="9" t="s">
         <v>295</v>
       </c>
-      <c r="E79" s="19" t="s">
+      <c r="E80" s="19" t="s">
         <v>296</v>
       </c>
-      <c r="F79" s="9" t="s">
+      <c r="F80" s="9" t="s">
         <v>298</v>
       </c>
-      <c r="G79" s="15" t="s">
+      <c r="G80" s="15" t="s">
         <v>401</v>
       </c>
-      <c r="H79" s="9" t="s">
+      <c r="H80" s="9" t="s">
         <v>297</v>
       </c>
-      <c r="I79" s="9"/>
-      <c r="J79" s="9"/>
+      <c r="I80" s="9"/>
+      <c r="J80" s="9"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1"/>

</xml_diff>